<commit_message>
FRM-42 kodunu hata önlemeye ayır; garanti formunu FRM-45 olarak düzelt
</commit_message>
<xml_diff>
--- a/EKG_Kalite_Yönetim_Sistemi/00_Yönetim Sistemi Çerçevesi/02_Doküman, Kayıt ve Kaynak Kontrolü/EKG-YNT-LST-02_Belge_Ana_Listesi.xlsx
+++ b/EKG_Kalite_Yönetim_Sistemi/00_Yönetim Sistemi Çerçevesi/02_Doküman, Kayıt ve Kaynak Kontrolü/EKG-YNT-LST-02_Belge_Ana_Listesi.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Gerekli Kaynak Kanıtları'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Klasör Anahtarları'!$A$1:$C$80</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Klasör Anahtarları'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Kontrol Özeti'!$A$1:$B$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Kontrol Özeti'!$A$1:$B$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Kontrol Özeti'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Ek Liste Kimlikleri'!$A$1:$G$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Ek Liste Kimlikleri'!$1:$1</definedName>
@@ -5952,7 +5952,7 @@
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>EKG-KLT-FRM-42</t>
+          <t>EKG-KLT-FRM-45</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
@@ -5967,7 +5967,7 @@
       </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t>EKG-KLT-FRM-42_garanti_on_analiz_kontrol_listesi_ve_raporu.xlsx</t>
+          <t>EKG-KLT-FRM-45_garanti_on_analiz_kontrol_listesi_ve_raporu.xlsx</t>
         </is>
       </c>
       <c r="E131" s="4" t="inlineStr">
@@ -5987,7 +5987,7 @@
       </c>
       <c r="H131" s="4" t="inlineStr">
         <is>
-          <t>Cam/pencere ön analizine uyarlandı; gözlem, kanıt ve yetkili garanti/ürün kararı ayrıldı.</t>
+          <t>Belge kodu FRM-42’den FRM-45’e taşındı; garanti ön analiz akışı korundu.</t>
         </is>
       </c>
     </row>
@@ -14456,7 +14456,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>EKG-KLT-FRM-42</t>
+          <t>EKG-KLT-FRM-45</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -14471,7 +14471,7 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>06_Garanti Sorunları Yönetimi/02_WIM2 - Ön Analiz, Kaynak ve Çevreleme/EKG-KLT-FRM-42_garanti_on_analiz_kontrol_listesi_ve_raporu.xlsx</t>
+          <t>06_Garanti Sorunları Yönetimi/02_WIM2 - Ön Analiz, Kaynak ve Çevreleme/EKG-KLT-FRM-45_garanti_on_analiz_kontrol_listesi_ve_raporu.xlsx</t>
         </is>
       </c>
     </row>
@@ -20206,12 +20206,12 @@
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>EKG-KLT-FRM-42</t>
+          <t>EKG-KLT-FRM-45</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>Cam/pencere ön analizine uyarlandı; gözlem, kanıt ve yetkili garanti/ürün kararı ayrıldı.</t>
+          <t>Önceki kod EKG-KLT-FRM-42. Cam/pencere ön analizine uyarlandı; gözlem, kanıt ve yetkili garanti/ürün kararı ayrıldı. Belge kodu, hata önleme formuyla çakışmayı gidermek için EKG-KLT-FRM-45 olarak değiştirildi.</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
@@ -20221,7 +20221,7 @@
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>Cam/pencere ön analizine uyarlandı; gözlem, kanıt ve yetkili garanti/ürün kararı ayrıldı.</t>
+          <t>Belge kodu FRM-42’den FRM-45’e taşındı; garanti ön analiz akışı korundu.</t>
         </is>
       </c>
     </row>
@@ -25477,7 +25477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -25643,53 +25643,65 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Gerekli kaynak kanıtları</t>
+          <t>Kapsama göre kod düzeltmesi</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>97 belge için müşteri/kuruluş kaynağı listelendi</t>
+          <t>EKG-KLT-FRM-42 → EKG-KLT-FRM-45</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Kayıt tarihleri</t>
+          <t>Gerekli kaynak kanıtları</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>İlk yayın/revizyon tarihleri belge kimliğidir; kaynak olay, test ve faaliyet tarihleri ayrı tutulur.</t>
+          <t>97 belge için müşteri/kuruluş kaynağı listelendi</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Tarih atama dayanağı</t>
+          <t>Kayıt tarihleri</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Kontrollü tarihler kullanıcı tarafından belirtilen aralıklara göre atanmıştır. Gerçek dosya güncelleme zamanı 19.10.2026 olarak korunmuştur.</t>
+          <t>İlk yayın/revizyon tarihleri belge kimliğidir; kaynak olay, test ve faaliyet tarihleri ayrı tutulur.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>Tarih atama dayanağı</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Kontrollü tarihler kullanıcı tarafından belirtilen aralıklara göre atanmıştır. Gerçek dosya güncelleme zamanı 19.10.2026 olarak korunmuştur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Kanıtların kullanımı</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Boş onaylar ve müşteri/kuruluş kanıtları doldurulmadı; gereken kaynaklar ilgili sayfada listelendi.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B17"/>
+  <autoFilter ref="A1:B18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" scale="100" fitToHeight="0" fitToWidth="0"/>
   <headerFooter>

</xml_diff>